<commit_message>
Mise à jour du category.display "Signes vitaux" remplacé par "vital-signs" dans Bp, Glucose and pain severity (#77)
* replace vital signs display

* update vital signs display

* add MS to device

* Revert "add MS to device"

This reverts commit 4e0c08421f0751e82620313f5c86b4c884ef4e6f. 35510c866b5ed6a8671dbb36d201efc78127b1ef
</commit_message>
<xml_diff>
--- a/ig/main/StructureDefinition-mesures-observation-glucose.xlsx
+++ b/ig/main/StructureDefinition-mesures-observation-glucose.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5061" uniqueCount="726">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5061" uniqueCount="725">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-11-28T13:27:45+00:00</t>
+    <t>2023-11-28T13:42:11+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1235,9 +1235,6 @@
   </si>
   <si>
     <t>Observation.category.coding.display</t>
-  </si>
-  <si>
-    <t>Signes vitaux</t>
   </si>
   <si>
     <t>Observation.category:VSCat.coding.userSelected</t>
@@ -8955,7 +8952,7 @@
         <v>81</v>
       </c>
       <c r="S53" t="s" s="2">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="T53" t="s" s="2">
         <v>81</v>
@@ -9029,10 +9026,10 @@
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
+        <v>391</v>
+      </c>
+      <c r="B54" t="s" s="2">
         <v>392</v>
-      </c>
-      <c r="B54" t="s" s="2">
-        <v>393</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -9151,10 +9148,10 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
+        <v>393</v>
+      </c>
+      <c r="B55" t="s" s="2">
         <v>394</v>
-      </c>
-      <c r="B55" t="s" s="2">
-        <v>395</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -9273,14 +9270,14 @@
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="E56" s="2"/>
       <c r="F56" t="s" s="2">
@@ -9302,16 +9299,16 @@
         <v>227</v>
       </c>
       <c r="L56" t="s" s="2">
+        <v>397</v>
+      </c>
+      <c r="M56" t="s" s="2">
         <v>398</v>
       </c>
-      <c r="M56" t="s" s="2">
+      <c r="N56" t="s" s="2">
         <v>399</v>
       </c>
-      <c r="N56" t="s" s="2">
+      <c r="O56" t="s" s="2">
         <v>400</v>
-      </c>
-      <c r="O56" t="s" s="2">
-        <v>401</v>
       </c>
       <c r="P56" t="s" s="2">
         <v>81</v>
@@ -9339,11 +9336,11 @@
         <v>152</v>
       </c>
       <c r="Y56" t="s" s="2">
+        <v>401</v>
+      </c>
+      <c r="Z56" t="s" s="2">
         <v>402</v>
       </c>
-      <c r="Z56" t="s" s="2">
-        <v>403</v>
-      </c>
       <c r="AA56" t="s" s="2">
         <v>81</v>
       </c>
@@ -9360,7 +9357,7 @@
         <v>81</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>92</v>
@@ -9375,30 +9372,30 @@
         <v>105</v>
       </c>
       <c r="AK56" t="s" s="2">
+        <v>403</v>
+      </c>
+      <c r="AL56" t="s" s="2">
         <v>404</v>
       </c>
-      <c r="AL56" t="s" s="2">
+      <c r="AM56" t="s" s="2">
         <v>405</v>
       </c>
-      <c r="AM56" t="s" s="2">
+      <c r="AN56" t="s" s="2">
         <v>406</v>
       </c>
-      <c r="AN56" t="s" s="2">
+      <c r="AO56" t="s" s="2">
         <v>407</v>
       </c>
-      <c r="AO56" t="s" s="2">
+      <c r="AP56" t="s" s="2">
         <v>408</v>
-      </c>
-      <c r="AP56" t="s" s="2">
-        <v>409</v>
       </c>
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -9513,10 +9510,10 @@
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -9633,10 +9630,10 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -9755,10 +9752,10 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -9873,10 +9870,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -9993,10 +9990,10 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -10115,10 +10112,10 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -10235,10 +10232,10 @@
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -10357,10 +10354,10 @@
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -10479,10 +10476,10 @@
     </row>
     <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -10601,10 +10598,10 @@
     </row>
     <row r="67" hidden="true">
       <c r="A67" t="s" s="2">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -10723,10 +10720,10 @@
     </row>
     <row r="68" hidden="true">
       <c r="A68" t="s" s="2">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -10749,19 +10746,19 @@
         <v>93</v>
       </c>
       <c r="K68" t="s" s="2">
+        <v>421</v>
+      </c>
+      <c r="L68" t="s" s="2">
         <v>422</v>
       </c>
-      <c r="L68" t="s" s="2">
+      <c r="M68" t="s" s="2">
         <v>423</v>
       </c>
-      <c r="M68" t="s" s="2">
+      <c r="N68" t="s" s="2">
         <v>424</v>
       </c>
-      <c r="N68" t="s" s="2">
+      <c r="O68" t="s" s="2">
         <v>425</v>
-      </c>
-      <c r="O68" t="s" s="2">
-        <v>426</v>
       </c>
       <c r="P68" t="s" s="2">
         <v>81</v>
@@ -10810,7 +10807,7 @@
         <v>81</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AG68" t="s" s="2">
         <v>79</v>
@@ -10825,19 +10822,19 @@
         <v>333</v>
       </c>
       <c r="AK68" t="s" s="2">
+        <v>426</v>
+      </c>
+      <c r="AL68" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM68" t="s" s="2">
         <v>427</v>
       </c>
-      <c r="AL68" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM68" t="s" s="2">
+      <c r="AN68" t="s" s="2">
         <v>428</v>
       </c>
-      <c r="AN68" t="s" s="2">
+      <c r="AO68" t="s" s="2">
         <v>429</v>
-      </c>
-      <c r="AO68" t="s" s="2">
-        <v>430</v>
       </c>
       <c r="AP68" t="s" s="2">
         <v>81</v>
@@ -10845,10 +10842,10 @@
     </row>
     <row r="69" hidden="true">
       <c r="A69" t="s" s="2">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -10871,16 +10868,16 @@
         <v>93</v>
       </c>
       <c r="K69" t="s" s="2">
+        <v>431</v>
+      </c>
+      <c r="L69" t="s" s="2">
         <v>432</v>
       </c>
-      <c r="L69" t="s" s="2">
+      <c r="M69" t="s" s="2">
         <v>433</v>
       </c>
-      <c r="M69" t="s" s="2">
+      <c r="N69" t="s" s="2">
         <v>434</v>
-      </c>
-      <c r="N69" t="s" s="2">
-        <v>435</v>
       </c>
       <c r="O69" s="2"/>
       <c r="P69" t="s" s="2">
@@ -10930,7 +10927,7 @@
         <v>81</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>79</v>
@@ -10951,13 +10948,13 @@
         <v>81</v>
       </c>
       <c r="AM69" t="s" s="2">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="AN69" t="s" s="2">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="AO69" t="s" s="2">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="AP69" t="s" s="2">
         <v>81</v>
@@ -10965,14 +10962,14 @@
     </row>
     <row r="70" hidden="true">
       <c r="A70" t="s" s="2">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="E70" s="2"/>
       <c r="F70" t="s" s="2">
@@ -10991,19 +10988,19 @@
         <v>93</v>
       </c>
       <c r="K70" t="s" s="2">
+        <v>438</v>
+      </c>
+      <c r="L70" t="s" s="2">
         <v>439</v>
       </c>
-      <c r="L70" t="s" s="2">
+      <c r="M70" t="s" s="2">
         <v>440</v>
       </c>
-      <c r="M70" t="s" s="2">
+      <c r="N70" t="s" s="2">
         <v>441</v>
       </c>
-      <c r="N70" t="s" s="2">
+      <c r="O70" t="s" s="2">
         <v>442</v>
-      </c>
-      <c r="O70" t="s" s="2">
-        <v>443</v>
       </c>
       <c r="P70" t="s" s="2">
         <v>81</v>
@@ -11052,7 +11049,7 @@
         <v>81</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>79</v>
@@ -11067,19 +11064,19 @@
         <v>333</v>
       </c>
       <c r="AK70" t="s" s="2">
+        <v>443</v>
+      </c>
+      <c r="AL70" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM70" t="s" s="2">
         <v>444</v>
       </c>
-      <c r="AL70" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM70" t="s" s="2">
+      <c r="AN70" t="s" s="2">
         <v>445</v>
       </c>
-      <c r="AN70" t="s" s="2">
+      <c r="AO70" t="s" s="2">
         <v>446</v>
-      </c>
-      <c r="AO70" t="s" s="2">
-        <v>447</v>
       </c>
       <c r="AP70" t="s" s="2">
         <v>81</v>
@@ -11087,14 +11084,14 @@
     </row>
     <row r="71" hidden="true">
       <c r="A71" t="s" s="2">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="E71" s="2"/>
       <c r="F71" t="s" s="2">
@@ -11113,19 +11110,19 @@
         <v>93</v>
       </c>
       <c r="K71" t="s" s="2">
+        <v>449</v>
+      </c>
+      <c r="L71" t="s" s="2">
         <v>450</v>
       </c>
-      <c r="L71" t="s" s="2">
+      <c r="M71" t="s" s="2">
         <v>451</v>
       </c>
-      <c r="M71" t="s" s="2">
+      <c r="N71" t="s" s="2">
         <v>452</v>
       </c>
-      <c r="N71" t="s" s="2">
+      <c r="O71" t="s" s="2">
         <v>453</v>
-      </c>
-      <c r="O71" t="s" s="2">
-        <v>454</v>
       </c>
       <c r="P71" t="s" s="2">
         <v>81</v>
@@ -11174,7 +11171,7 @@
         <v>81</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>79</v>
@@ -11183,25 +11180,25 @@
         <v>92</v>
       </c>
       <c r="AI71" t="s" s="2">
+        <v>454</v>
+      </c>
+      <c r="AJ71" t="s" s="2">
         <v>455</v>
       </c>
-      <c r="AJ71" t="s" s="2">
+      <c r="AK71" t="s" s="2">
         <v>456</v>
       </c>
-      <c r="AK71" t="s" s="2">
+      <c r="AL71" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM71" t="s" s="2">
         <v>457</v>
       </c>
-      <c r="AL71" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM71" t="s" s="2">
+      <c r="AN71" t="s" s="2">
         <v>458</v>
       </c>
-      <c r="AN71" t="s" s="2">
+      <c r="AO71" t="s" s="2">
         <v>459</v>
-      </c>
-      <c r="AO71" t="s" s="2">
-        <v>460</v>
       </c>
       <c r="AP71" t="s" s="2">
         <v>81</v>
@@ -11209,10 +11206,10 @@
     </row>
     <row r="72" hidden="true">
       <c r="A72" t="s" s="2">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -11238,13 +11235,13 @@
         <v>130</v>
       </c>
       <c r="L72" t="s" s="2">
+        <v>461</v>
+      </c>
+      <c r="M72" t="s" s="2">
         <v>462</v>
       </c>
-      <c r="M72" t="s" s="2">
+      <c r="N72" t="s" s="2">
         <v>463</v>
-      </c>
-      <c r="N72" t="s" s="2">
-        <v>464</v>
       </c>
       <c r="O72" s="2"/>
       <c r="P72" t="s" s="2">
@@ -11294,7 +11291,7 @@
         <v>81</v>
       </c>
       <c r="AF72" t="s" s="2">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="AG72" t="s" s="2">
         <v>79</v>
@@ -11315,13 +11312,13 @@
         <v>81</v>
       </c>
       <c r="AM72" t="s" s="2">
+        <v>464</v>
+      </c>
+      <c r="AN72" t="s" s="2">
         <v>465</v>
       </c>
-      <c r="AN72" t="s" s="2">
+      <c r="AO72" t="s" s="2">
         <v>466</v>
-      </c>
-      <c r="AO72" t="s" s="2">
-        <v>467</v>
       </c>
       <c r="AP72" t="s" s="2">
         <v>81</v>
@@ -11329,10 +11326,10 @@
     </row>
     <row r="73" hidden="true">
       <c r="A73" t="s" s="2">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -11355,19 +11352,19 @@
         <v>93</v>
       </c>
       <c r="K73" t="s" s="2">
+        <v>468</v>
+      </c>
+      <c r="L73" t="s" s="2">
         <v>469</v>
       </c>
-      <c r="L73" t="s" s="2">
+      <c r="M73" t="s" s="2">
         <v>470</v>
-      </c>
-      <c r="M73" t="s" s="2">
-        <v>471</v>
       </c>
       <c r="N73" t="s" s="2">
         <v>331</v>
       </c>
       <c r="O73" t="s" s="2">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="P73" t="s" s="2">
         <v>81</v>
@@ -11416,7 +11413,7 @@
         <v>81</v>
       </c>
       <c r="AF73" t="s" s="2">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="AG73" t="s" s="2">
         <v>79</v>
@@ -11431,19 +11428,19 @@
         <v>333</v>
       </c>
       <c r="AK73" t="s" s="2">
+        <v>472</v>
+      </c>
+      <c r="AL73" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM73" t="s" s="2">
         <v>473</v>
       </c>
-      <c r="AL73" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM73" t="s" s="2">
+      <c r="AN73" t="s" s="2">
         <v>474</v>
       </c>
-      <c r="AN73" t="s" s="2">
+      <c r="AO73" t="s" s="2">
         <v>475</v>
-      </c>
-      <c r="AO73" t="s" s="2">
-        <v>476</v>
       </c>
       <c r="AP73" t="s" s="2">
         <v>81</v>
@@ -11451,10 +11448,10 @@
     </row>
     <row r="74" hidden="true">
       <c r="A74" t="s" s="2">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -11477,19 +11474,19 @@
         <v>93</v>
       </c>
       <c r="K74" t="s" s="2">
+        <v>477</v>
+      </c>
+      <c r="L74" t="s" s="2">
         <v>478</v>
       </c>
-      <c r="L74" t="s" s="2">
+      <c r="M74" t="s" s="2">
+        <v>478</v>
+      </c>
+      <c r="N74" t="s" s="2">
         <v>479</v>
       </c>
-      <c r="M74" t="s" s="2">
-        <v>479</v>
-      </c>
-      <c r="N74" t="s" s="2">
+      <c r="O74" t="s" s="2">
         <v>480</v>
-      </c>
-      <c r="O74" t="s" s="2">
-        <v>481</v>
       </c>
       <c r="P74" t="s" s="2">
         <v>81</v>
@@ -11538,7 +11535,7 @@
         <v>81</v>
       </c>
       <c r="AF74" t="s" s="2">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="AG74" t="s" s="2">
         <v>79</v>
@@ -11547,7 +11544,7 @@
         <v>92</v>
       </c>
       <c r="AI74" t="s" s="2">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="AJ74" t="s" s="2">
         <v>105</v>
@@ -11556,27 +11553,27 @@
         <v>81</v>
       </c>
       <c r="AL74" t="s" s="2">
+        <v>482</v>
+      </c>
+      <c r="AM74" t="s" s="2">
         <v>483</v>
       </c>
-      <c r="AM74" t="s" s="2">
+      <c r="AN74" t="s" s="2">
         <v>484</v>
       </c>
-      <c r="AN74" t="s" s="2">
+      <c r="AO74" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AP74" t="s" s="2">
         <v>485</v>
-      </c>
-      <c r="AO74" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AP74" t="s" s="2">
-        <v>486</v>
       </c>
     </row>
     <row r="75" hidden="true">
       <c r="A75" t="s" s="2">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
@@ -11691,10 +11688,10 @@
     </row>
     <row r="76" hidden="true">
       <c r="A76" t="s" s="2">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -11811,10 +11808,10 @@
     </row>
     <row r="77" hidden="true">
       <c r="A77" t="s" s="2">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -11837,19 +11834,19 @@
         <v>93</v>
       </c>
       <c r="K77" t="s" s="2">
+        <v>489</v>
+      </c>
+      <c r="L77" t="s" s="2">
         <v>490</v>
       </c>
-      <c r="L77" t="s" s="2">
+      <c r="M77" t="s" s="2">
         <v>491</v>
       </c>
-      <c r="M77" t="s" s="2">
+      <c r="N77" t="s" s="2">
         <v>492</v>
       </c>
-      <c r="N77" t="s" s="2">
+      <c r="O77" t="s" s="2">
         <v>493</v>
-      </c>
-      <c r="O77" t="s" s="2">
-        <v>494</v>
       </c>
       <c r="P77" t="s" s="2">
         <v>81</v>
@@ -11898,7 +11895,7 @@
         <v>81</v>
       </c>
       <c r="AF77" t="s" s="2">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>79</v>
@@ -11919,10 +11916,10 @@
         <v>81</v>
       </c>
       <c r="AM77" t="s" s="2">
+        <v>495</v>
+      </c>
+      <c r="AN77" t="s" s="2">
         <v>496</v>
-      </c>
-      <c r="AN77" t="s" s="2">
-        <v>497</v>
       </c>
       <c r="AO77" t="s" s="2">
         <v>81</v>
@@ -11933,10 +11930,10 @@
     </row>
     <row r="78" hidden="true">
       <c r="A78" t="s" s="2">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -11962,22 +11959,22 @@
         <v>172</v>
       </c>
       <c r="L78" t="s" s="2">
+        <v>498</v>
+      </c>
+      <c r="M78" t="s" s="2">
         <v>499</v>
-      </c>
-      <c r="M78" t="s" s="2">
-        <v>500</v>
       </c>
       <c r="N78" t="s" s="2">
         <v>271</v>
       </c>
       <c r="O78" t="s" s="2">
+        <v>500</v>
+      </c>
+      <c r="P78" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q78" t="s" s="2">
         <v>501</v>
-      </c>
-      <c r="P78" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Q78" t="s" s="2">
-        <v>502</v>
       </c>
       <c r="R78" t="s" s="2">
         <v>81</v>
@@ -12001,28 +11998,28 @@
         <v>230</v>
       </c>
       <c r="Y78" t="s" s="2">
+        <v>502</v>
+      </c>
+      <c r="Z78" t="s" s="2">
         <v>503</v>
       </c>
-      <c r="Z78" t="s" s="2">
+      <c r="AA78" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB78" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC78" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD78" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE78" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF78" t="s" s="2">
         <v>504</v>
-      </c>
-      <c r="AA78" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AB78" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AC78" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AD78" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AE78" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AF78" t="s" s="2">
-        <v>505</v>
       </c>
       <c r="AG78" t="s" s="2">
         <v>79</v>
@@ -12043,10 +12040,10 @@
         <v>81</v>
       </c>
       <c r="AM78" t="s" s="2">
+        <v>505</v>
+      </c>
+      <c r="AN78" t="s" s="2">
         <v>506</v>
-      </c>
-      <c r="AN78" t="s" s="2">
-        <v>507</v>
       </c>
       <c r="AO78" t="s" s="2">
         <v>81</v>
@@ -12057,10 +12054,10 @@
     </row>
     <row r="79" hidden="true">
       <c r="A79" t="s" s="2">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -12086,16 +12083,16 @@
         <v>108</v>
       </c>
       <c r="L79" t="s" s="2">
+        <v>508</v>
+      </c>
+      <c r="M79" t="s" s="2">
         <v>509</v>
-      </c>
-      <c r="M79" t="s" s="2">
-        <v>510</v>
       </c>
       <c r="N79" t="s" s="2">
         <v>271</v>
       </c>
       <c r="O79" t="s" s="2">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="P79" t="s" s="2">
         <v>81</v>
@@ -12144,7 +12141,7 @@
         <v>81</v>
       </c>
       <c r="AF79" t="s" s="2">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="AG79" t="s" s="2">
         <v>79</v>
@@ -12165,10 +12162,10 @@
         <v>81</v>
       </c>
       <c r="AM79" t="s" s="2">
+        <v>512</v>
+      </c>
+      <c r="AN79" t="s" s="2">
         <v>513</v>
-      </c>
-      <c r="AN79" t="s" s="2">
-        <v>514</v>
       </c>
       <c r="AO79" t="s" s="2">
         <v>81</v>
@@ -12179,10 +12176,10 @@
     </row>
     <row r="80" hidden="true">
       <c r="A80" t="s" s="2">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -12208,16 +12205,16 @@
         <v>136</v>
       </c>
       <c r="L80" t="s" s="2">
+        <v>515</v>
+      </c>
+      <c r="M80" t="s" s="2">
         <v>516</v>
       </c>
-      <c r="M80" t="s" s="2">
+      <c r="N80" t="s" s="2">
         <v>517</v>
       </c>
-      <c r="N80" t="s" s="2">
+      <c r="O80" t="s" s="2">
         <v>518</v>
-      </c>
-      <c r="O80" t="s" s="2">
-        <v>519</v>
       </c>
       <c r="P80" t="s" s="2">
         <v>81</v>
@@ -12227,55 +12224,55 @@
         <v>81</v>
       </c>
       <c r="S80" t="s" s="2">
+        <v>519</v>
+      </c>
+      <c r="T80" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U80" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V80" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W80" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X80" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y80" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z80" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA80" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB80" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC80" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD80" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE80" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF80" t="s" s="2">
         <v>520</v>
       </c>
-      <c r="T80" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="U80" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="V80" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="W80" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="X80" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Y80" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Z80" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AA80" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AB80" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AC80" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AD80" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AE80" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AF80" t="s" s="2">
+      <c r="AG80" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH80" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="AI80" t="s" s="2">
         <v>521</v>
-      </c>
-      <c r="AG80" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH80" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="AI80" t="s" s="2">
-        <v>522</v>
       </c>
       <c r="AJ80" t="s" s="2">
         <v>105</v>
@@ -12287,10 +12284,10 @@
         <v>81</v>
       </c>
       <c r="AM80" t="s" s="2">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="AN80" t="s" s="2">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="AO80" t="s" s="2">
         <v>81</v>
@@ -12301,10 +12298,10 @@
     </row>
     <row r="81" hidden="true">
       <c r="A81" t="s" s="2">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -12330,16 +12327,16 @@
         <v>172</v>
       </c>
       <c r="L81" t="s" s="2">
+        <v>524</v>
+      </c>
+      <c r="M81" t="s" s="2">
         <v>525</v>
       </c>
-      <c r="M81" t="s" s="2">
+      <c r="N81" t="s" s="2">
         <v>526</v>
       </c>
-      <c r="N81" t="s" s="2">
+      <c r="O81" t="s" s="2">
         <v>527</v>
-      </c>
-      <c r="O81" t="s" s="2">
-        <v>528</v>
       </c>
       <c r="P81" t="s" s="2">
         <v>81</v>
@@ -12367,28 +12364,28 @@
         <v>230</v>
       </c>
       <c r="Y81" t="s" s="2">
+        <v>528</v>
+      </c>
+      <c r="Z81" t="s" s="2">
+        <v>528</v>
+      </c>
+      <c r="AA81" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB81" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC81" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD81" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE81" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF81" t="s" s="2">
         <v>529</v>
-      </c>
-      <c r="Z81" t="s" s="2">
-        <v>529</v>
-      </c>
-      <c r="AA81" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AB81" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AC81" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AD81" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AE81" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AF81" t="s" s="2">
-        <v>530</v>
       </c>
       <c r="AG81" t="s" s="2">
         <v>79</v>
@@ -12409,10 +12406,10 @@
         <v>81</v>
       </c>
       <c r="AM81" t="s" s="2">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="AN81" t="s" s="2">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="AO81" t="s" s="2">
         <v>81</v>
@@ -12423,10 +12420,10 @@
     </row>
     <row r="82" hidden="true">
       <c r="A82" t="s" s="2">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -12452,16 +12449,16 @@
         <v>227</v>
       </c>
       <c r="L82" t="s" s="2">
+        <v>532</v>
+      </c>
+      <c r="M82" t="s" s="2">
         <v>533</v>
       </c>
-      <c r="M82" t="s" s="2">
+      <c r="N82" t="s" s="2">
         <v>534</v>
       </c>
-      <c r="N82" t="s" s="2">
+      <c r="O82" t="s" s="2">
         <v>535</v>
-      </c>
-      <c r="O82" t="s" s="2">
-        <v>536</v>
       </c>
       <c r="P82" t="s" s="2">
         <v>81</v>
@@ -12489,37 +12486,37 @@
         <v>152</v>
       </c>
       <c r="Y82" t="s" s="2">
+        <v>536</v>
+      </c>
+      <c r="Z82" t="s" s="2">
         <v>537</v>
       </c>
-      <c r="Z82" t="s" s="2">
+      <c r="AA82" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB82" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC82" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD82" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE82" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF82" t="s" s="2">
+        <v>531</v>
+      </c>
+      <c r="AG82" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH82" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="AI82" t="s" s="2">
         <v>538</v>
-      </c>
-      <c r="AA82" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AB82" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AC82" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AD82" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AE82" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AF82" t="s" s="2">
-        <v>532</v>
-      </c>
-      <c r="AG82" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH82" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="AI82" t="s" s="2">
-        <v>539</v>
       </c>
       <c r="AJ82" t="s" s="2">
         <v>105</v>
@@ -12534,7 +12531,7 @@
         <v>106</v>
       </c>
       <c r="AN82" t="s" s="2">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="AO82" t="s" s="2">
         <v>81</v>
@@ -12545,10 +12542,10 @@
     </row>
     <row r="83" hidden="true">
       <c r="A83" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -12663,10 +12660,10 @@
     </row>
     <row r="84" hidden="true">
       <c r="A84" t="s" s="2">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -12783,10 +12780,10 @@
     </row>
     <row r="85" hidden="true">
       <c r="A85" t="s" s="2">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -12905,10 +12902,10 @@
     </row>
     <row r="86" hidden="true">
       <c r="A86" t="s" s="2">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -13023,10 +13020,10 @@
     </row>
     <row r="87" hidden="true">
       <c r="A87" t="s" s="2">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -13143,10 +13140,10 @@
     </row>
     <row r="88" hidden="true">
       <c r="A88" t="s" s="2">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -13265,10 +13262,10 @@
     </row>
     <row r="89" hidden="true">
       <c r="A89" t="s" s="2">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -13385,10 +13382,10 @@
     </row>
     <row r="90" hidden="true">
       <c r="A90" t="s" s="2">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -13507,10 +13504,10 @@
     </row>
     <row r="91" hidden="true">
       <c r="A91" t="s" s="2">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -13629,10 +13626,10 @@
     </row>
     <row r="92" hidden="true">
       <c r="A92" t="s" s="2">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -13751,10 +13748,10 @@
     </row>
     <row r="93" hidden="true">
       <c r="A93" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -13873,14 +13870,14 @@
     </row>
     <row r="94" hidden="true">
       <c r="A94" t="s" s="2">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="E94" s="2"/>
       <c r="F94" t="s" s="2">
@@ -13902,16 +13899,16 @@
         <v>227</v>
       </c>
       <c r="L94" t="s" s="2">
+        <v>553</v>
+      </c>
+      <c r="M94" t="s" s="2">
         <v>554</v>
       </c>
-      <c r="M94" t="s" s="2">
+      <c r="N94" t="s" s="2">
         <v>555</v>
       </c>
-      <c r="N94" t="s" s="2">
+      <c r="O94" t="s" s="2">
         <v>556</v>
-      </c>
-      <c r="O94" t="s" s="2">
-        <v>557</v>
       </c>
       <c r="P94" t="s" s="2">
         <v>81</v>
@@ -13939,11 +13936,11 @@
         <v>152</v>
       </c>
       <c r="Y94" t="s" s="2">
+        <v>557</v>
+      </c>
+      <c r="Z94" t="s" s="2">
         <v>558</v>
       </c>
-      <c r="Z94" t="s" s="2">
-        <v>559</v>
-      </c>
       <c r="AA94" t="s" s="2">
         <v>81</v>
       </c>
@@ -13960,7 +13957,7 @@
         <v>81</v>
       </c>
       <c r="AF94" t="s" s="2">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="AG94" t="s" s="2">
         <v>79</v>
@@ -13978,27 +13975,27 @@
         <v>81</v>
       </c>
       <c r="AL94" t="s" s="2">
+        <v>559</v>
+      </c>
+      <c r="AM94" t="s" s="2">
         <v>560</v>
       </c>
-      <c r="AM94" t="s" s="2">
+      <c r="AN94" t="s" s="2">
         <v>561</v>
       </c>
-      <c r="AN94" t="s" s="2">
+      <c r="AO94" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AP94" t="s" s="2">
         <v>562</v>
-      </c>
-      <c r="AO94" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AP94" t="s" s="2">
-        <v>563</v>
       </c>
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -14021,19 +14018,19 @@
         <v>81</v>
       </c>
       <c r="K95" t="s" s="2">
+        <v>564</v>
+      </c>
+      <c r="L95" t="s" s="2">
         <v>565</v>
       </c>
-      <c r="L95" t="s" s="2">
+      <c r="M95" t="s" s="2">
         <v>566</v>
       </c>
-      <c r="M95" t="s" s="2">
+      <c r="N95" t="s" s="2">
         <v>567</v>
       </c>
-      <c r="N95" t="s" s="2">
+      <c r="O95" t="s" s="2">
         <v>568</v>
-      </c>
-      <c r="O95" t="s" s="2">
-        <v>569</v>
       </c>
       <c r="P95" t="s" s="2">
         <v>81</v>
@@ -14082,7 +14079,7 @@
         <v>81</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>79</v>
@@ -14103,10 +14100,10 @@
         <v>81</v>
       </c>
       <c r="AM95" t="s" s="2">
+        <v>569</v>
+      </c>
+      <c r="AN95" t="s" s="2">
         <v>570</v>
-      </c>
-      <c r="AN95" t="s" s="2">
-        <v>571</v>
       </c>
       <c r="AO95" t="s" s="2">
         <v>81</v>
@@ -14117,10 +14114,10 @@
     </row>
     <row r="96" hidden="true">
       <c r="A96" t="s" s="2">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -14146,13 +14143,13 @@
         <v>227</v>
       </c>
       <c r="L96" t="s" s="2">
+        <v>572</v>
+      </c>
+      <c r="M96" t="s" s="2">
         <v>573</v>
       </c>
-      <c r="M96" t="s" s="2">
+      <c r="N96" t="s" s="2">
         <v>574</v>
-      </c>
-      <c r="N96" t="s" s="2">
-        <v>575</v>
       </c>
       <c r="O96" s="2"/>
       <c r="P96" t="s" s="2">
@@ -14181,11 +14178,11 @@
         <v>162</v>
       </c>
       <c r="Y96" t="s" s="2">
+        <v>575</v>
+      </c>
+      <c r="Z96" t="s" s="2">
         <v>576</v>
       </c>
-      <c r="Z96" t="s" s="2">
-        <v>577</v>
-      </c>
       <c r="AA96" t="s" s="2">
         <v>81</v>
       </c>
@@ -14202,7 +14199,7 @@
         <v>81</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>79</v>
@@ -14220,27 +14217,27 @@
         <v>81</v>
       </c>
       <c r="AL96" t="s" s="2">
+        <v>577</v>
+      </c>
+      <c r="AM96" t="s" s="2">
         <v>578</v>
       </c>
-      <c r="AM96" t="s" s="2">
+      <c r="AN96" t="s" s="2">
         <v>579</v>
       </c>
-      <c r="AN96" t="s" s="2">
+      <c r="AO96" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AP96" t="s" s="2">
         <v>580</v>
-      </c>
-      <c r="AO96" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AP96" t="s" s="2">
-        <v>581</v>
       </c>
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -14266,16 +14263,16 @@
         <v>227</v>
       </c>
       <c r="L97" t="s" s="2">
+        <v>582</v>
+      </c>
+      <c r="M97" t="s" s="2">
         <v>583</v>
       </c>
-      <c r="M97" t="s" s="2">
+      <c r="N97" t="s" s="2">
         <v>584</v>
       </c>
-      <c r="N97" t="s" s="2">
+      <c r="O97" t="s" s="2">
         <v>585</v>
-      </c>
-      <c r="O97" t="s" s="2">
-        <v>586</v>
       </c>
       <c r="P97" t="s" s="2">
         <v>81</v>
@@ -14304,7 +14301,7 @@
       </c>
       <c r="Y97" s="2"/>
       <c r="Z97" t="s" s="2">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="AA97" t="s" s="2">
         <v>81</v>
@@ -14322,7 +14319,7 @@
         <v>81</v>
       </c>
       <c r="AF97" t="s" s="2">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="AG97" t="s" s="2">
         <v>79</v>
@@ -14343,10 +14340,10 @@
         <v>81</v>
       </c>
       <c r="AM97" t="s" s="2">
+        <v>587</v>
+      </c>
+      <c r="AN97" t="s" s="2">
         <v>588</v>
-      </c>
-      <c r="AN97" t="s" s="2">
-        <v>589</v>
       </c>
       <c r="AO97" t="s" s="2">
         <v>81</v>
@@ -14357,10 +14354,10 @@
     </row>
     <row r="98" hidden="true">
       <c r="A98" t="s" s="2">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -14383,16 +14380,16 @@
         <v>81</v>
       </c>
       <c r="K98" t="s" s="2">
+        <v>590</v>
+      </c>
+      <c r="L98" t="s" s="2">
         <v>591</v>
       </c>
-      <c r="L98" t="s" s="2">
+      <c r="M98" t="s" s="2">
         <v>592</v>
       </c>
-      <c r="M98" t="s" s="2">
+      <c r="N98" t="s" s="2">
         <v>593</v>
-      </c>
-      <c r="N98" t="s" s="2">
-        <v>594</v>
       </c>
       <c r="O98" s="2"/>
       <c r="P98" t="s" s="2">
@@ -14442,7 +14439,7 @@
         <v>81</v>
       </c>
       <c r="AF98" t="s" s="2">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="AG98" t="s" s="2">
         <v>79</v>
@@ -14460,27 +14457,27 @@
         <v>81</v>
       </c>
       <c r="AL98" t="s" s="2">
+        <v>594</v>
+      </c>
+      <c r="AM98" t="s" s="2">
         <v>595</v>
       </c>
-      <c r="AM98" t="s" s="2">
+      <c r="AN98" t="s" s="2">
         <v>596</v>
       </c>
-      <c r="AN98" t="s" s="2">
+      <c r="AO98" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AP98" t="s" s="2">
         <v>597</v>
-      </c>
-      <c r="AO98" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AP98" t="s" s="2">
-        <v>598</v>
       </c>
     </row>
     <row r="99" hidden="true">
       <c r="A99" t="s" s="2">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -14503,16 +14500,16 @@
         <v>81</v>
       </c>
       <c r="K99" t="s" s="2">
+        <v>599</v>
+      </c>
+      <c r="L99" t="s" s="2">
         <v>600</v>
       </c>
-      <c r="L99" t="s" s="2">
+      <c r="M99" t="s" s="2">
         <v>601</v>
       </c>
-      <c r="M99" t="s" s="2">
+      <c r="N99" t="s" s="2">
         <v>602</v>
-      </c>
-      <c r="N99" t="s" s="2">
-        <v>603</v>
       </c>
       <c r="O99" s="2"/>
       <c r="P99" t="s" s="2">
@@ -14562,7 +14559,7 @@
         <v>81</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>79</v>
@@ -14580,27 +14577,27 @@
         <v>81</v>
       </c>
       <c r="AL99" t="s" s="2">
+        <v>603</v>
+      </c>
+      <c r="AM99" t="s" s="2">
         <v>604</v>
       </c>
-      <c r="AM99" t="s" s="2">
+      <c r="AN99" t="s" s="2">
         <v>605</v>
       </c>
-      <c r="AN99" t="s" s="2">
+      <c r="AO99" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AP99" t="s" s="2">
         <v>606</v>
-      </c>
-      <c r="AO99" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AP99" t="s" s="2">
-        <v>607</v>
       </c>
     </row>
     <row r="100" hidden="true">
       <c r="A100" t="s" s="2">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -14623,19 +14620,19 @@
         <v>81</v>
       </c>
       <c r="K100" t="s" s="2">
+        <v>608</v>
+      </c>
+      <c r="L100" t="s" s="2">
         <v>609</v>
       </c>
-      <c r="L100" t="s" s="2">
+      <c r="M100" t="s" s="2">
         <v>610</v>
       </c>
-      <c r="M100" t="s" s="2">
+      <c r="N100" t="s" s="2">
         <v>611</v>
       </c>
-      <c r="N100" t="s" s="2">
+      <c r="O100" t="s" s="2">
         <v>612</v>
-      </c>
-      <c r="O100" t="s" s="2">
-        <v>613</v>
       </c>
       <c r="P100" t="s" s="2">
         <v>81</v>
@@ -14684,7 +14681,7 @@
         <v>81</v>
       </c>
       <c r="AF100" t="s" s="2">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>79</v>
@@ -14696,19 +14693,19 @@
         <v>104</v>
       </c>
       <c r="AJ100" t="s" s="2">
+        <v>613</v>
+      </c>
+      <c r="AK100" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL100" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM100" t="s" s="2">
         <v>614</v>
       </c>
-      <c r="AK100" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL100" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM100" t="s" s="2">
+      <c r="AN100" t="s" s="2">
         <v>615</v>
-      </c>
-      <c r="AN100" t="s" s="2">
-        <v>616</v>
       </c>
       <c r="AO100" t="s" s="2">
         <v>81</v>
@@ -14719,10 +14716,10 @@
     </row>
     <row r="101" hidden="true">
       <c r="A101" t="s" s="2">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -14837,10 +14834,10 @@
     </row>
     <row r="102" hidden="true">
       <c r="A102" t="s" s="2">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -14957,14 +14954,14 @@
     </row>
     <row r="103" hidden="true">
       <c r="A103" t="s" s="2">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="E103" s="2"/>
       <c r="F103" t="s" s="2">
@@ -14986,10 +14983,10 @@
         <v>115</v>
       </c>
       <c r="L103" t="s" s="2">
+        <v>620</v>
+      </c>
+      <c r="M103" t="s" s="2">
         <v>621</v>
-      </c>
-      <c r="M103" t="s" s="2">
-        <v>622</v>
       </c>
       <c r="N103" t="s" s="2">
         <v>118</v>
@@ -15044,7 +15041,7 @@
         <v>81</v>
       </c>
       <c r="AF103" t="s" s="2">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="AG103" t="s" s="2">
         <v>79</v>
@@ -15079,10 +15076,10 @@
     </row>
     <row r="104" hidden="true">
       <c r="A104" t="s" s="2">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -15105,16 +15102,16 @@
         <v>81</v>
       </c>
       <c r="K104" t="s" s="2">
+        <v>624</v>
+      </c>
+      <c r="L104" t="s" s="2">
         <v>625</v>
       </c>
-      <c r="L104" t="s" s="2">
+      <c r="M104" t="s" s="2">
         <v>626</v>
       </c>
-      <c r="M104" t="s" s="2">
+      <c r="N104" t="s" s="2">
         <v>627</v>
-      </c>
-      <c r="N104" t="s" s="2">
-        <v>628</v>
       </c>
       <c r="O104" s="2"/>
       <c r="P104" t="s" s="2">
@@ -15164,7 +15161,7 @@
         <v>81</v>
       </c>
       <c r="AF104" t="s" s="2">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="AG104" t="s" s="2">
         <v>79</v>
@@ -15173,22 +15170,22 @@
         <v>92</v>
       </c>
       <c r="AI104" t="s" s="2">
+        <v>628</v>
+      </c>
+      <c r="AJ104" t="s" s="2">
         <v>629</v>
       </c>
-      <c r="AJ104" t="s" s="2">
+      <c r="AK104" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL104" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM104" t="s" s="2">
         <v>630</v>
       </c>
-      <c r="AK104" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL104" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM104" t="s" s="2">
+      <c r="AN104" t="s" s="2">
         <v>631</v>
-      </c>
-      <c r="AN104" t="s" s="2">
-        <v>632</v>
       </c>
       <c r="AO104" t="s" s="2">
         <v>81</v>
@@ -15199,10 +15196,10 @@
     </row>
     <row r="105" hidden="true">
       <c r="A105" t="s" s="2">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" t="s" s="2">
@@ -15225,16 +15222,16 @@
         <v>81</v>
       </c>
       <c r="K105" t="s" s="2">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="L105" t="s" s="2">
+        <v>633</v>
+      </c>
+      <c r="M105" t="s" s="2">
         <v>634</v>
       </c>
-      <c r="M105" t="s" s="2">
-        <v>635</v>
-      </c>
       <c r="N105" t="s" s="2">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="O105" s="2"/>
       <c r="P105" t="s" s="2">
@@ -15284,7 +15281,7 @@
         <v>81</v>
       </c>
       <c r="AF105" t="s" s="2">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="AG105" t="s" s="2">
         <v>79</v>
@@ -15293,22 +15290,22 @@
         <v>92</v>
       </c>
       <c r="AI105" t="s" s="2">
+        <v>628</v>
+      </c>
+      <c r="AJ105" t="s" s="2">
         <v>629</v>
       </c>
-      <c r="AJ105" t="s" s="2">
+      <c r="AK105" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL105" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM105" t="s" s="2">
         <v>630</v>
       </c>
-      <c r="AK105" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL105" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM105" t="s" s="2">
-        <v>631</v>
-      </c>
       <c r="AN105" t="s" s="2">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="AO105" t="s" s="2">
         <v>81</v>
@@ -15319,10 +15316,10 @@
     </row>
     <row r="106" hidden="true">
       <c r="A106" t="s" s="2">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" t="s" s="2">
@@ -15348,16 +15345,16 @@
         <v>227</v>
       </c>
       <c r="L106" t="s" s="2">
+        <v>637</v>
+      </c>
+      <c r="M106" t="s" s="2">
         <v>638</v>
       </c>
-      <c r="M106" t="s" s="2">
+      <c r="N106" t="s" s="2">
         <v>639</v>
       </c>
-      <c r="N106" t="s" s="2">
+      <c r="O106" t="s" s="2">
         <v>640</v>
-      </c>
-      <c r="O106" t="s" s="2">
-        <v>641</v>
       </c>
       <c r="P106" t="s" s="2">
         <v>81</v>
@@ -15385,11 +15382,11 @@
         <v>176</v>
       </c>
       <c r="Y106" t="s" s="2">
+        <v>641</v>
+      </c>
+      <c r="Z106" t="s" s="2">
         <v>642</v>
       </c>
-      <c r="Z106" t="s" s="2">
-        <v>643</v>
-      </c>
       <c r="AA106" t="s" s="2">
         <v>81</v>
       </c>
@@ -15406,7 +15403,7 @@
         <v>81</v>
       </c>
       <c r="AF106" t="s" s="2">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="AG106" t="s" s="2">
         <v>79</v>
@@ -15424,13 +15421,13 @@
         <v>81</v>
       </c>
       <c r="AL106" t="s" s="2">
+        <v>643</v>
+      </c>
+      <c r="AM106" t="s" s="2">
         <v>644</v>
       </c>
-      <c r="AM106" t="s" s="2">
-        <v>645</v>
-      </c>
       <c r="AN106" t="s" s="2">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="AO106" t="s" s="2">
         <v>81</v>
@@ -15441,10 +15438,10 @@
     </row>
     <row r="107" hidden="true">
       <c r="A107" t="s" s="2">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" t="s" s="2">
@@ -15470,16 +15467,16 @@
         <v>227</v>
       </c>
       <c r="L107" t="s" s="2">
+        <v>646</v>
+      </c>
+      <c r="M107" t="s" s="2">
         <v>647</v>
       </c>
-      <c r="M107" t="s" s="2">
+      <c r="N107" t="s" s="2">
         <v>648</v>
       </c>
-      <c r="N107" t="s" s="2">
+      <c r="O107" t="s" s="2">
         <v>649</v>
-      </c>
-      <c r="O107" t="s" s="2">
-        <v>650</v>
       </c>
       <c r="P107" t="s" s="2">
         <v>81</v>
@@ -15507,11 +15504,11 @@
         <v>230</v>
       </c>
       <c r="Y107" t="s" s="2">
+        <v>650</v>
+      </c>
+      <c r="Z107" t="s" s="2">
         <v>651</v>
       </c>
-      <c r="Z107" t="s" s="2">
-        <v>652</v>
-      </c>
       <c r="AA107" t="s" s="2">
         <v>81</v>
       </c>
@@ -15528,7 +15525,7 @@
         <v>81</v>
       </c>
       <c r="AF107" t="s" s="2">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="AG107" t="s" s="2">
         <v>79</v>
@@ -15546,13 +15543,13 @@
         <v>81</v>
       </c>
       <c r="AL107" t="s" s="2">
+        <v>643</v>
+      </c>
+      <c r="AM107" t="s" s="2">
         <v>644</v>
       </c>
-      <c r="AM107" t="s" s="2">
-        <v>645</v>
-      </c>
       <c r="AN107" t="s" s="2">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="AO107" t="s" s="2">
         <v>81</v>
@@ -15563,10 +15560,10 @@
     </row>
     <row r="108" hidden="true">
       <c r="A108" t="s" s="2">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" t="s" s="2">
@@ -15681,10 +15678,10 @@
     </row>
     <row r="109" hidden="true">
       <c r="A109" t="s" s="2">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" t="s" s="2">
@@ -15801,10 +15798,10 @@
     </row>
     <row r="110" hidden="true">
       <c r="A110" t="s" s="2">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" t="s" s="2">
@@ -15923,10 +15920,10 @@
     </row>
     <row r="111" hidden="true">
       <c r="A111" t="s" s="2">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B111" t="s" s="2">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="C111" s="2"/>
       <c r="D111" t="s" s="2">
@@ -16041,10 +16038,10 @@
     </row>
     <row r="112" hidden="true">
       <c r="A112" t="s" s="2">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B112" t="s" s="2">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" t="s" s="2">
@@ -16161,10 +16158,10 @@
     </row>
     <row r="113" hidden="true">
       <c r="A113" t="s" s="2">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="B113" t="s" s="2">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" t="s" s="2">
@@ -16283,10 +16280,10 @@
     </row>
     <row r="114" hidden="true">
       <c r="A114" t="s" s="2">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B114" t="s" s="2">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" t="s" s="2">
@@ -16403,10 +16400,10 @@
     </row>
     <row r="115" hidden="true">
       <c r="A115" t="s" s="2">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B115" t="s" s="2">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="C115" s="2"/>
       <c r="D115" t="s" s="2">
@@ -16525,10 +16522,10 @@
     </row>
     <row r="116" hidden="true">
       <c r="A116" t="s" s="2">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="B116" t="s" s="2">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" t="s" s="2">
@@ -16647,10 +16644,10 @@
     </row>
     <row r="117" hidden="true">
       <c r="A117" t="s" s="2">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B117" t="s" s="2">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C117" s="2"/>
       <c r="D117" t="s" s="2">
@@ -16769,10 +16766,10 @@
     </row>
     <row r="118" hidden="true">
       <c r="A118" t="s" s="2">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B118" t="s" s="2">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="C118" s="2"/>
       <c r="D118" t="s" s="2">
@@ -16891,10 +16888,10 @@
     </row>
     <row r="119" hidden="true">
       <c r="A119" t="s" s="2">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B119" t="s" s="2">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="C119" s="2"/>
       <c r="D119" t="s" s="2">
@@ -16917,19 +16914,19 @@
         <v>81</v>
       </c>
       <c r="K119" t="s" s="2">
+        <v>664</v>
+      </c>
+      <c r="L119" t="s" s="2">
         <v>665</v>
       </c>
-      <c r="L119" t="s" s="2">
+      <c r="M119" t="s" s="2">
         <v>666</v>
       </c>
-      <c r="M119" t="s" s="2">
+      <c r="N119" t="s" s="2">
         <v>667</v>
       </c>
-      <c r="N119" t="s" s="2">
+      <c r="O119" t="s" s="2">
         <v>668</v>
-      </c>
-      <c r="O119" t="s" s="2">
-        <v>669</v>
       </c>
       <c r="P119" t="s" s="2">
         <v>81</v>
@@ -16978,7 +16975,7 @@
         <v>81</v>
       </c>
       <c r="AF119" t="s" s="2">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="AG119" t="s" s="2">
         <v>79</v>
@@ -16990,19 +16987,19 @@
         <v>104</v>
       </c>
       <c r="AJ119" t="s" s="2">
+        <v>669</v>
+      </c>
+      <c r="AK119" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL119" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM119" t="s" s="2">
         <v>670</v>
       </c>
-      <c r="AK119" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL119" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM119" t="s" s="2">
+      <c r="AN119" t="s" s="2">
         <v>671</v>
-      </c>
-      <c r="AN119" t="s" s="2">
-        <v>672</v>
       </c>
       <c r="AO119" t="s" s="2">
         <v>81</v>
@@ -17013,10 +17010,10 @@
     </row>
     <row r="120" hidden="true">
       <c r="A120" t="s" s="2">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B120" t="s" s="2">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="C120" s="2"/>
       <c r="D120" t="s" s="2">
@@ -17042,10 +17039,10 @@
         <v>108</v>
       </c>
       <c r="L120" t="s" s="2">
+        <v>673</v>
+      </c>
+      <c r="M120" t="s" s="2">
         <v>674</v>
-      </c>
-      <c r="M120" t="s" s="2">
-        <v>675</v>
       </c>
       <c r="N120" t="s" s="2">
         <v>271</v>
@@ -17098,7 +17095,7 @@
         <v>81</v>
       </c>
       <c r="AF120" t="s" s="2">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="AG120" t="s" s="2">
         <v>79</v>
@@ -17119,10 +17116,10 @@
         <v>81</v>
       </c>
       <c r="AM120" t="s" s="2">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="AN120" t="s" s="2">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="AO120" t="s" s="2">
         <v>81</v>
@@ -17133,10 +17130,10 @@
     </row>
     <row r="121" hidden="true">
       <c r="A121" t="s" s="2">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B121" t="s" s="2">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="C121" s="2"/>
       <c r="D121" t="s" s="2">
@@ -17159,16 +17156,16 @@
         <v>93</v>
       </c>
       <c r="K121" t="s" s="2">
+        <v>677</v>
+      </c>
+      <c r="L121" t="s" s="2">
         <v>678</v>
       </c>
-      <c r="L121" t="s" s="2">
+      <c r="M121" t="s" s="2">
         <v>679</v>
       </c>
-      <c r="M121" t="s" s="2">
+      <c r="N121" t="s" s="2">
         <v>680</v>
-      </c>
-      <c r="N121" t="s" s="2">
-        <v>681</v>
       </c>
       <c r="O121" s="2"/>
       <c r="P121" t="s" s="2">
@@ -17218,7 +17215,7 @@
         <v>81</v>
       </c>
       <c r="AF121" t="s" s="2">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="AG121" t="s" s="2">
         <v>79</v>
@@ -17239,10 +17236,10 @@
         <v>81</v>
       </c>
       <c r="AM121" t="s" s="2">
+        <v>681</v>
+      </c>
+      <c r="AN121" t="s" s="2">
         <v>682</v>
-      </c>
-      <c r="AN121" t="s" s="2">
-        <v>683</v>
       </c>
       <c r="AO121" t="s" s="2">
         <v>81</v>
@@ -17253,10 +17250,10 @@
     </row>
     <row r="122" hidden="true">
       <c r="A122" t="s" s="2">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="B122" t="s" s="2">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="C122" s="2"/>
       <c r="D122" t="s" s="2">
@@ -17279,16 +17276,16 @@
         <v>93</v>
       </c>
       <c r="K122" t="s" s="2">
+        <v>684</v>
+      </c>
+      <c r="L122" t="s" s="2">
         <v>685</v>
       </c>
-      <c r="L122" t="s" s="2">
+      <c r="M122" t="s" s="2">
         <v>686</v>
       </c>
-      <c r="M122" t="s" s="2">
+      <c r="N122" t="s" s="2">
         <v>687</v>
-      </c>
-      <c r="N122" t="s" s="2">
-        <v>688</v>
       </c>
       <c r="O122" s="2"/>
       <c r="P122" t="s" s="2">
@@ -17338,7 +17335,7 @@
         <v>81</v>
       </c>
       <c r="AF122" t="s" s="2">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="AG122" t="s" s="2">
         <v>79</v>
@@ -17359,10 +17356,10 @@
         <v>81</v>
       </c>
       <c r="AM122" t="s" s="2">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="AN122" t="s" s="2">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="AO122" t="s" s="2">
         <v>81</v>
@@ -17373,10 +17370,10 @@
     </row>
     <row r="123" hidden="true">
       <c r="A123" t="s" s="2">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="B123" t="s" s="2">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="C123" s="2"/>
       <c r="D123" t="s" s="2">
@@ -17399,19 +17396,19 @@
         <v>93</v>
       </c>
       <c r="K123" t="s" s="2">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="L123" t="s" s="2">
+        <v>690</v>
+      </c>
+      <c r="M123" t="s" s="2">
+        <v>690</v>
+      </c>
+      <c r="N123" t="s" s="2">
         <v>691</v>
       </c>
-      <c r="M123" t="s" s="2">
-        <v>691</v>
-      </c>
-      <c r="N123" t="s" s="2">
+      <c r="O123" t="s" s="2">
         <v>692</v>
-      </c>
-      <c r="O123" t="s" s="2">
-        <v>693</v>
       </c>
       <c r="P123" t="s" s="2">
         <v>81</v>
@@ -17460,7 +17457,7 @@
         <v>81</v>
       </c>
       <c r="AF123" t="s" s="2">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="AG123" t="s" s="2">
         <v>79</v>
@@ -17472,19 +17469,19 @@
         <v>104</v>
       </c>
       <c r="AJ123" t="s" s="2">
+        <v>693</v>
+      </c>
+      <c r="AK123" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL123" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM123" t="s" s="2">
         <v>694</v>
       </c>
-      <c r="AK123" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL123" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM123" t="s" s="2">
+      <c r="AN123" t="s" s="2">
         <v>695</v>
-      </c>
-      <c r="AN123" t="s" s="2">
-        <v>696</v>
       </c>
       <c r="AO123" t="s" s="2">
         <v>81</v>
@@ -17495,10 +17492,10 @@
     </row>
     <row r="124" hidden="true">
       <c r="A124" t="s" s="2">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="B124" t="s" s="2">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" t="s" s="2">
@@ -17613,10 +17610,10 @@
     </row>
     <row r="125" hidden="true">
       <c r="A125" t="s" s="2">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="B125" t="s" s="2">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="C125" s="2"/>
       <c r="D125" t="s" s="2">
@@ -17733,14 +17730,14 @@
     </row>
     <row r="126" hidden="true">
       <c r="A126" t="s" s="2">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="B126" t="s" s="2">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C126" s="2"/>
       <c r="D126" t="s" s="2">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="E126" s="2"/>
       <c r="F126" t="s" s="2">
@@ -17762,10 +17759,10 @@
         <v>115</v>
       </c>
       <c r="L126" t="s" s="2">
+        <v>620</v>
+      </c>
+      <c r="M126" t="s" s="2">
         <v>621</v>
-      </c>
-      <c r="M126" t="s" s="2">
-        <v>622</v>
       </c>
       <c r="N126" t="s" s="2">
         <v>118</v>
@@ -17820,7 +17817,7 @@
         <v>81</v>
       </c>
       <c r="AF126" t="s" s="2">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="AG126" t="s" s="2">
         <v>79</v>
@@ -17855,10 +17852,10 @@
     </row>
     <row r="127" hidden="true">
       <c r="A127" t="s" s="2">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="B127" t="s" s="2">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="C127" s="2"/>
       <c r="D127" t="s" s="2">
@@ -17884,16 +17881,16 @@
         <v>227</v>
       </c>
       <c r="L127" t="s" s="2">
+        <v>700</v>
+      </c>
+      <c r="M127" t="s" s="2">
         <v>701</v>
       </c>
-      <c r="M127" t="s" s="2">
+      <c r="N127" t="s" s="2">
         <v>702</v>
       </c>
-      <c r="N127" t="s" s="2">
+      <c r="O127" t="s" s="2">
         <v>703</v>
-      </c>
-      <c r="O127" t="s" s="2">
-        <v>704</v>
       </c>
       <c r="P127" t="s" s="2">
         <v>81</v>
@@ -17921,11 +17918,11 @@
         <v>152</v>
       </c>
       <c r="Y127" t="s" s="2">
+        <v>704</v>
+      </c>
+      <c r="Z127" t="s" s="2">
         <v>705</v>
       </c>
-      <c r="Z127" t="s" s="2">
-        <v>706</v>
-      </c>
       <c r="AA127" t="s" s="2">
         <v>81</v>
       </c>
@@ -17942,7 +17939,7 @@
         <v>81</v>
       </c>
       <c r="AF127" t="s" s="2">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="AG127" t="s" s="2">
         <v>92</v>
@@ -17960,16 +17957,16 @@
         <v>81</v>
       </c>
       <c r="AL127" t="s" s="2">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="AM127" t="s" s="2">
+        <v>405</v>
+      </c>
+      <c r="AN127" t="s" s="2">
         <v>406</v>
       </c>
-      <c r="AN127" t="s" s="2">
+      <c r="AO127" t="s" s="2">
         <v>407</v>
-      </c>
-      <c r="AO127" t="s" s="2">
-        <v>408</v>
       </c>
       <c r="AP127" t="s" s="2">
         <v>81</v>
@@ -17977,10 +17974,10 @@
     </row>
     <row r="128" hidden="true">
       <c r="A128" t="s" s="2">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B128" t="s" s="2">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="C128" s="2"/>
       <c r="D128" t="s" s="2">
@@ -18003,19 +18000,19 @@
         <v>93</v>
       </c>
       <c r="K128" t="s" s="2">
+        <v>708</v>
+      </c>
+      <c r="L128" t="s" s="2">
         <v>709</v>
       </c>
-      <c r="L128" t="s" s="2">
+      <c r="M128" t="s" s="2">
         <v>710</v>
       </c>
-      <c r="M128" t="s" s="2">
+      <c r="N128" t="s" s="2">
         <v>711</v>
       </c>
-      <c r="N128" t="s" s="2">
-        <v>712</v>
-      </c>
       <c r="O128" t="s" s="2">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="P128" t="s" s="2">
         <v>81</v>
@@ -18043,37 +18040,37 @@
         <v>230</v>
       </c>
       <c r="Y128" t="s" s="2">
+        <v>712</v>
+      </c>
+      <c r="Z128" t="s" s="2">
         <v>713</v>
       </c>
-      <c r="Z128" t="s" s="2">
+      <c r="AA128" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB128" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC128" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD128" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE128" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF128" t="s" s="2">
+        <v>707</v>
+      </c>
+      <c r="AG128" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH128" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="AI128" t="s" s="2">
         <v>714</v>
-      </c>
-      <c r="AA128" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AB128" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AC128" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AD128" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AE128" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AF128" t="s" s="2">
-        <v>708</v>
-      </c>
-      <c r="AG128" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH128" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="AI128" t="s" s="2">
-        <v>715</v>
       </c>
       <c r="AJ128" t="s" s="2">
         <v>105</v>
@@ -18082,27 +18079,27 @@
         <v>81</v>
       </c>
       <c r="AL128" t="s" s="2">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="AM128" t="s" s="2">
+        <v>483</v>
+      </c>
+      <c r="AN128" t="s" s="2">
         <v>484</v>
       </c>
-      <c r="AN128" t="s" s="2">
+      <c r="AO128" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AP128" t="s" s="2">
         <v>485</v>
-      </c>
-      <c r="AO128" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AP128" t="s" s="2">
-        <v>486</v>
       </c>
     </row>
     <row r="129" hidden="true">
       <c r="A129" t="s" s="2">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="B129" t="s" s="2">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="C129" s="2"/>
       <c r="D129" t="s" s="2">
@@ -18128,16 +18125,16 @@
         <v>227</v>
       </c>
       <c r="L129" t="s" s="2">
+        <v>717</v>
+      </c>
+      <c r="M129" t="s" s="2">
         <v>718</v>
       </c>
-      <c r="M129" t="s" s="2">
+      <c r="N129" t="s" s="2">
         <v>719</v>
       </c>
-      <c r="N129" t="s" s="2">
-        <v>720</v>
-      </c>
       <c r="O129" t="s" s="2">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="P129" t="s" s="2">
         <v>81</v>
@@ -18165,11 +18162,11 @@
         <v>152</v>
       </c>
       <c r="Y129" t="s" s="2">
+        <v>536</v>
+      </c>
+      <c r="Z129" t="s" s="2">
         <v>537</v>
       </c>
-      <c r="Z129" t="s" s="2">
-        <v>538</v>
-      </c>
       <c r="AA129" t="s" s="2">
         <v>81</v>
       </c>
@@ -18186,7 +18183,7 @@
         <v>81</v>
       </c>
       <c r="AF129" t="s" s="2">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="AG129" t="s" s="2">
         <v>79</v>
@@ -18195,7 +18192,7 @@
         <v>92</v>
       </c>
       <c r="AI129" t="s" s="2">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="AJ129" t="s" s="2">
         <v>105</v>
@@ -18210,7 +18207,7 @@
         <v>106</v>
       </c>
       <c r="AN129" t="s" s="2">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="AO129" t="s" s="2">
         <v>81</v>
@@ -18221,14 +18218,14 @@
     </row>
     <row r="130" hidden="true">
       <c r="A130" t="s" s="2">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="B130" t="s" s="2">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="C130" s="2"/>
       <c r="D130" t="s" s="2">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="E130" s="2"/>
       <c r="F130" t="s" s="2">
@@ -18250,16 +18247,16 @@
         <v>227</v>
       </c>
       <c r="L130" t="s" s="2">
+        <v>553</v>
+      </c>
+      <c r="M130" t="s" s="2">
         <v>554</v>
       </c>
-      <c r="M130" t="s" s="2">
+      <c r="N130" t="s" s="2">
         <v>555</v>
       </c>
-      <c r="N130" t="s" s="2">
+      <c r="O130" t="s" s="2">
         <v>556</v>
-      </c>
-      <c r="O130" t="s" s="2">
-        <v>557</v>
       </c>
       <c r="P130" t="s" s="2">
         <v>81</v>
@@ -18287,11 +18284,11 @@
         <v>152</v>
       </c>
       <c r="Y130" t="s" s="2">
+        <v>557</v>
+      </c>
+      <c r="Z130" t="s" s="2">
         <v>558</v>
       </c>
-      <c r="Z130" t="s" s="2">
-        <v>559</v>
-      </c>
       <c r="AA130" t="s" s="2">
         <v>81</v>
       </c>
@@ -18308,7 +18305,7 @@
         <v>81</v>
       </c>
       <c r="AF130" t="s" s="2">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="AG130" t="s" s="2">
         <v>79</v>
@@ -18326,27 +18323,27 @@
         <v>81</v>
       </c>
       <c r="AL130" t="s" s="2">
+        <v>559</v>
+      </c>
+      <c r="AM130" t="s" s="2">
         <v>560</v>
       </c>
-      <c r="AM130" t="s" s="2">
+      <c r="AN130" t="s" s="2">
         <v>561</v>
       </c>
-      <c r="AN130" t="s" s="2">
+      <c r="AO130" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AP130" t="s" s="2">
         <v>562</v>
-      </c>
-      <c r="AO130" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AP130" t="s" s="2">
-        <v>563</v>
       </c>
     </row>
     <row r="131" hidden="true">
       <c r="A131" t="s" s="2">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B131" t="s" s="2">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="C131" s="2"/>
       <c r="D131" t="s" s="2">
@@ -18372,16 +18369,16 @@
         <v>82</v>
       </c>
       <c r="L131" t="s" s="2">
+        <v>723</v>
+      </c>
+      <c r="M131" t="s" s="2">
         <v>724</v>
       </c>
-      <c r="M131" t="s" s="2">
-        <v>725</v>
-      </c>
       <c r="N131" t="s" s="2">
+        <v>611</v>
+      </c>
+      <c r="O131" t="s" s="2">
         <v>612</v>
-      </c>
-      <c r="O131" t="s" s="2">
-        <v>613</v>
       </c>
       <c r="P131" t="s" s="2">
         <v>81</v>
@@ -18430,7 +18427,7 @@
         <v>81</v>
       </c>
       <c r="AF131" t="s" s="2">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="AG131" t="s" s="2">
         <v>79</v>
@@ -18451,10 +18448,10 @@
         <v>81</v>
       </c>
       <c r="AM131" t="s" s="2">
+        <v>614</v>
+      </c>
+      <c r="AN131" t="s" s="2">
         <v>615</v>
-      </c>
-      <c r="AN131" t="s" s="2">
-        <v>616</v>
       </c>
       <c r="AO131" t="s" s="2">
         <v>81</v>

</xml_diff>